<commit_message>
Stabilize OA pipeline package, notebooks, tests, and docs
</commit_message>
<xml_diff>
--- a/examples/example_data.xlsx
+++ b/examples/example_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="oa_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="oa_data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -644,37 +644,37 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>45374</v>
+        <v>45352</v>
       </c>
       <c r="I2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2" t="n">
-        <v>5.548377302761811</v>
+        <v>5.548704057043798</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5489770328343222</v>
+        <v>0.5529323495133089</v>
       </c>
       <c r="L2" t="n">
-        <v>33.81</v>
+        <v>33.08</v>
       </c>
       <c r="M2" t="n">
-        <v>25.9</v>
+        <v>24.35</v>
       </c>
       <c r="N2" t="n">
-        <v>25.51</v>
+        <v>24.41</v>
       </c>
       <c r="O2" t="n">
-        <v>17.19</v>
+        <v>11.92</v>
       </c>
       <c r="P2" t="n">
-        <v>2335.12</v>
+        <v>2254.38</v>
       </c>
       <c r="Q2" t="n">
-        <v>8.041</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="R2" t="n">
-        <v>8.042</v>
+        <v>8.034000000000001</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -687,16 +687,16 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>2132.78</v>
+        <v>2060.48</v>
       </c>
       <c r="V2" t="n">
-        <v>24.47</v>
+        <v>17.62</v>
       </c>
       <c r="W2" t="n">
-        <v>1977.32</v>
+        <v>1909.57</v>
       </c>
       <c r="X2" t="n">
-        <v>130.99</v>
+        <v>133.29</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -727,28 +727,28 @@
         </is>
       </c>
       <c r="AE2" t="n">
-        <v>194.6</v>
+        <v>219.3</v>
       </c>
       <c r="AF2" t="n">
-        <v>5.41</v>
+        <v>7.27</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.982</v>
+        <v>0.656</v>
       </c>
       <c r="AH2" t="n">
-        <v>10.6</v>
+        <v>4.32</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.95</v>
+        <v>3.85</v>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -789,37 +789,37 @@
         </is>
       </c>
       <c r="H3" s="1" t="n">
-        <v>45366</v>
+        <v>45353</v>
       </c>
       <c r="I3" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>5.60156890055749</v>
+        <v>5.602233684019246</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6000542037503458</v>
+        <v>0.5999722783693459</v>
       </c>
       <c r="L3" t="n">
-        <v>34.35</v>
+        <v>34.68</v>
       </c>
       <c r="M3" t="n">
-        <v>28.59</v>
+        <v>27.9</v>
       </c>
       <c r="N3" t="n">
-        <v>28.46</v>
+        <v>28.4</v>
       </c>
       <c r="O3" t="n">
-        <v>23.11</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="P3" t="n">
-        <v>2345.29</v>
+        <v>2237.14</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.978</v>
+        <v>7.966</v>
       </c>
       <c r="R3" t="n">
-        <v>7.969</v>
+        <v>7.972</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -832,16 +832,16 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>2081.97</v>
+        <v>2025.98</v>
       </c>
       <c r="V3" t="n">
-        <v>17.25</v>
+        <v>19.23</v>
       </c>
       <c r="W3" t="n">
-        <v>1899.33</v>
+        <v>1886.12</v>
       </c>
       <c r="X3" t="n">
-        <v>165.39</v>
+        <v>120.63</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="AC3" t="n">
-        <v>470.9</v>
+        <v>426.1</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
@@ -872,28 +872,28 @@
         </is>
       </c>
       <c r="AE3" t="n">
-        <v>206.1</v>
+        <v>231.8</v>
       </c>
       <c r="AF3" t="n">
-        <v>6.97</v>
+        <v>7.43</v>
       </c>
       <c r="AG3" t="n">
-        <v>1.14</v>
+        <v>0.076</v>
       </c>
       <c r="AH3" t="n">
-        <v>13.95</v>
+        <v>6.73</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.67</v>
+        <v>4.39</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -934,37 +934,37 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>45405</v>
+        <v>45354</v>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J4" t="n">
-        <v>5.653117639921701</v>
+        <v>5.648683197038944</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6491842265836193</v>
+        <v>0.6477858619193597</v>
       </c>
       <c r="L4" t="n">
-        <v>34.09</v>
+        <v>34.15</v>
       </c>
       <c r="M4" t="n">
-        <v>27.03</v>
+        <v>27.55</v>
       </c>
       <c r="N4" t="n">
-        <v>27.06</v>
+        <v>27.55</v>
       </c>
       <c r="O4" t="n">
-        <v>14.04</v>
+        <v>13.57</v>
       </c>
       <c r="P4" t="n">
-        <v>2324.59</v>
+        <v>2256.87</v>
       </c>
       <c r="Q4" t="n">
-        <v>8.002000000000001</v>
+        <v>8.118</v>
       </c>
       <c r="R4" t="n">
-        <v>8.003</v>
+        <v>8.109</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -977,16 +977,16 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>2128.06</v>
+        <v>2022.9</v>
       </c>
       <c r="V4" t="n">
-        <v>14.18</v>
+        <v>22.79</v>
       </c>
       <c r="W4" t="n">
-        <v>1994.93</v>
+        <v>1908.63</v>
       </c>
       <c r="X4" t="n">
-        <v>118.95</v>
+        <v>91.48</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="AC4" t="n">
-        <v>450.3</v>
+        <v>409.9</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
@@ -1017,28 +1017,28 @@
         </is>
       </c>
       <c r="AE4" t="n">
-        <v>235.2</v>
+        <v>215.6</v>
       </c>
       <c r="AF4" t="n">
-        <v>4.45</v>
+        <v>7.85</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.256</v>
+        <v>0.164</v>
       </c>
       <c r="AH4" t="n">
-        <v>11.88</v>
+        <v>7.54</v>
       </c>
       <c r="AI4" t="n">
-        <v>4.15</v>
+        <v>1.88</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1079,37 +1079,37 @@
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>45370</v>
+        <v>45355</v>
       </c>
       <c r="I5" t="n">
         <v>20</v>
       </c>
       <c r="J5" t="n">
-        <v>5.703098212879543</v>
+        <v>5.701134796083317</v>
       </c>
       <c r="K5" t="n">
-        <v>0.698173305830031</v>
+        <v>0.6974648105369891</v>
       </c>
       <c r="L5" t="n">
-        <v>34.33</v>
+        <v>33.06</v>
       </c>
       <c r="M5" t="n">
-        <v>27.32</v>
+        <v>25.46</v>
       </c>
       <c r="N5" t="n">
-        <v>27.18</v>
+        <v>25.65</v>
       </c>
       <c r="O5" t="n">
-        <v>10.83</v>
+        <v>5.59</v>
       </c>
       <c r="P5" t="n">
-        <v>2229.06</v>
+        <v>2341.48</v>
       </c>
       <c r="Q5" t="n">
-        <v>8.071999999999999</v>
+        <v>8.125999999999999</v>
       </c>
       <c r="R5" t="n">
-        <v>8.073</v>
+        <v>8.119</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1122,16 +1122,16 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>2021.2</v>
+        <v>2109.37</v>
       </c>
       <c r="V5" t="n">
-        <v>18.16</v>
+        <v>18.08</v>
       </c>
       <c r="W5" t="n">
-        <v>1919.67</v>
+        <v>1980.54</v>
       </c>
       <c r="X5" t="n">
-        <v>83.37</v>
+        <v>110.75</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>480.3</v>
+        <v>444.3</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
@@ -1162,28 +1162,28 @@
         </is>
       </c>
       <c r="AE5" t="n">
-        <v>236.2</v>
+        <v>239</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.67</v>
+        <v>2.68</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.469</v>
+        <v>0.232</v>
       </c>
       <c r="AH5" t="n">
-        <v>13.35</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="AI5" t="n">
-        <v>3.17</v>
+        <v>1.9</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1224,37 +1224,37 @@
         </is>
       </c>
       <c r="H6" s="1" t="n">
-        <v>45374</v>
+        <v>45356</v>
       </c>
       <c r="I6" t="n">
         <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>5.550864371747913</v>
+        <v>5.547154266433813</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5527108357763126</v>
+        <v>0.5511107159032274</v>
       </c>
       <c r="L6" t="n">
         <v>50</v>
       </c>
       <c r="M6" t="n">
-        <v>27.44</v>
+        <v>23.92</v>
       </c>
       <c r="N6" t="n">
-        <v>27.19</v>
+        <v>24.13</v>
       </c>
       <c r="O6" t="n">
-        <v>7.73</v>
+        <v>2.33</v>
       </c>
       <c r="P6" t="n">
-        <v>2211.05</v>
+        <v>2212.71</v>
       </c>
       <c r="Q6" t="n">
-        <v>8.141</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="R6" t="n">
-        <v>8.148999999999999</v>
+        <v>8.038</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1267,16 +1267,16 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>1980.87</v>
+        <v>2012.91</v>
       </c>
       <c r="V6" t="n">
-        <v>11.96</v>
+        <v>10.56</v>
       </c>
       <c r="W6" t="n">
-        <v>1820.55</v>
+        <v>1918.92</v>
       </c>
       <c r="X6" t="n">
-        <v>148.36</v>
+        <v>83.43000000000001</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="AC6" t="n">
-        <v>441.5</v>
+        <v>451.4</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
@@ -1307,28 +1307,28 @@
         </is>
       </c>
       <c r="AE6" t="n">
-        <v>239</v>
+        <v>236.6</v>
       </c>
       <c r="AF6" t="n">
-        <v>1.24</v>
+        <v>2.8</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.54</v>
+        <v>0.519</v>
       </c>
       <c r="AH6" t="n">
-        <v>6.54</v>
+        <v>2.64</v>
       </c>
       <c r="AI6" t="n">
-        <v>4.82</v>
+        <v>4.77</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1369,37 +1369,37 @@
         </is>
       </c>
       <c r="H7" s="1" t="n">
-        <v>45372</v>
+        <v>45357</v>
       </c>
       <c r="I7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J7" t="n">
-        <v>5.599274657534936</v>
+        <v>5.599219764398573</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5999951360052959</v>
+        <v>0.6023602285801135</v>
       </c>
       <c r="L7" t="n">
-        <v>35.82</v>
+        <v>34.78</v>
       </c>
       <c r="M7" t="n">
-        <v>28.26</v>
+        <v>23.86</v>
       </c>
       <c r="N7" t="n">
-        <v>28.47</v>
+        <v>24.21</v>
       </c>
       <c r="O7" t="n">
-        <v>14.33</v>
+        <v>9.43</v>
       </c>
       <c r="P7" t="n">
-        <v>2295.45</v>
+        <v>2212.39</v>
       </c>
       <c r="Q7" t="n">
-        <v>8.117000000000001</v>
+        <v>8.015000000000001</v>
       </c>
       <c r="R7" t="n">
-        <v>8.122</v>
+        <v>8.023</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1412,16 +1412,16 @@
         </is>
       </c>
       <c r="U7" t="n">
-        <v>2109.02</v>
+        <v>1975.31</v>
       </c>
       <c r="V7" t="n">
-        <v>18.65</v>
+        <v>11.56</v>
       </c>
       <c r="W7" t="n">
-        <v>1977.78</v>
+        <v>1862.65</v>
       </c>
       <c r="X7" t="n">
-        <v>112.59</v>
+        <v>101.1</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="AC7" t="n">
-        <v>497.5</v>
+        <v>481.5</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
@@ -1452,28 +1452,28 @@
         </is>
       </c>
       <c r="AE7" t="n">
-        <v>204.6</v>
+        <v>220.3</v>
       </c>
       <c r="AF7" t="n">
-        <v>1.68</v>
+        <v>4.89</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.702</v>
+        <v>0.826</v>
       </c>
       <c r="AH7" t="n">
-        <v>6.61</v>
+        <v>13.87</v>
       </c>
       <c r="AI7" t="n">
-        <v>2.97</v>
+        <v>3.12</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1510,37 +1510,37 @@
         </is>
       </c>
       <c r="H8" s="1" t="n">
-        <v>45411</v>
+        <v>45358</v>
       </c>
       <c r="I8" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J8" t="n">
-        <v>5.647843494896325</v>
+        <v>5.650256077764607</v>
       </c>
       <c r="K8" t="n">
-        <v>0.651638155136534</v>
+        <v>0.6510138154015482</v>
       </c>
       <c r="L8" t="n">
-        <v>34.57</v>
+        <v>33.87</v>
       </c>
       <c r="M8" t="n">
-        <v>25.01</v>
+        <v>27.43</v>
       </c>
       <c r="N8" t="n">
-        <v>25</v>
+        <v>26.94</v>
       </c>
       <c r="O8" t="n">
-        <v>15.69</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>2303.65</v>
+        <v>2209.79</v>
       </c>
       <c r="Q8" t="n">
-        <v>8.045</v>
+        <v>7.96</v>
       </c>
       <c r="R8" t="n">
-        <v>8.050000000000001</v>
+        <v>7.958</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1553,16 +1553,16 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>2111.79</v>
+        <v>1992</v>
       </c>
       <c r="V8" t="n">
-        <v>19.7</v>
+        <v>21.39</v>
       </c>
       <c r="W8" t="n">
-        <v>1943.24</v>
+        <v>1878.35</v>
       </c>
       <c r="X8" t="n">
-        <v>148.85</v>
+        <v>92.26000000000001</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="AC8" t="n">
-        <v>491.7</v>
+        <v>434</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
@@ -1593,28 +1593,28 @@
         </is>
       </c>
       <c r="AE8" t="n">
-        <v>205.3</v>
+        <v>203.1</v>
       </c>
       <c r="AF8" t="n">
-        <v>3.56</v>
+        <v>6.11</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.107</v>
+        <v>0.877</v>
       </c>
       <c r="AH8" t="n">
-        <v>14.38</v>
+        <v>8.68</v>
       </c>
       <c r="AI8" t="n">
-        <v>1.33</v>
+        <v>1.47</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1655,37 +1655,37 @@
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>45409</v>
+        <v>45359</v>
       </c>
       <c r="I9" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J9" t="n">
-        <v>5.699689096762078</v>
+        <v>5.703042021722376</v>
       </c>
       <c r="K9" t="n">
-        <v>0.701576438730213</v>
+        <v>0.7009149305220952</v>
       </c>
       <c r="L9" t="n">
-        <v>34.16</v>
+        <v>34.05</v>
       </c>
       <c r="M9" t="n">
-        <v>28.68</v>
+        <v>26.33</v>
       </c>
       <c r="N9" t="n">
-        <v>28.87</v>
+        <v>26.05</v>
       </c>
       <c r="O9" t="n">
-        <v>21.46</v>
+        <v>3.21</v>
       </c>
       <c r="P9" t="n">
-        <v>2277.49</v>
+        <v>2322.39</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.003</v>
+        <v>8.036</v>
       </c>
       <c r="R9" t="n">
-        <v>8.01</v>
+        <v>8.044</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1698,16 +1698,16 @@
         </is>
       </c>
       <c r="U9" t="n">
-        <v>2090.22</v>
+        <v>2106.55</v>
       </c>
       <c r="V9" t="n">
-        <v>20.94</v>
+        <v>18.46</v>
       </c>
       <c r="W9" t="n">
-        <v>1973.22</v>
+        <v>1925.95</v>
       </c>
       <c r="X9" t="n">
-        <v>96.06</v>
+        <v>162.14</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -1730,7 +1730,7 @@
         </is>
       </c>
       <c r="AC9" t="n">
-        <v>452.7</v>
+        <v>478.7</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
@@ -1738,28 +1738,28 @@
         </is>
       </c>
       <c r="AE9" t="n">
-        <v>219.3</v>
+        <v>200.8</v>
       </c>
       <c r="AF9" t="n">
-        <v>5.56</v>
+        <v>1.92</v>
       </c>
       <c r="AG9" t="n">
-        <v>1.1</v>
+        <v>0.599</v>
       </c>
       <c r="AH9" t="n">
-        <v>9.92</v>
+        <v>2.8</v>
       </c>
       <c r="AI9" t="n">
-        <v>2.56</v>
+        <v>3.23</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1800,37 +1800,37 @@
         </is>
       </c>
       <c r="H10" s="1" t="n">
-        <v>45364</v>
+        <v>45360</v>
       </c>
       <c r="I10" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J10" t="n">
-        <v>5.548638105903003</v>
+        <v>5.548377302761811</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5501601379967801</v>
+        <v>0.5489770328343222</v>
       </c>
       <c r="L10" t="n">
-        <v>35.96</v>
+        <v>33.81</v>
       </c>
       <c r="M10" t="n">
-        <v>26.85</v>
+        <v>25.9</v>
       </c>
       <c r="N10" t="n">
-        <v>26.81</v>
+        <v>25.51</v>
       </c>
       <c r="O10" t="n">
-        <v>12.35</v>
+        <v>23.64</v>
       </c>
       <c r="P10" t="n">
-        <v>2261.61</v>
+        <v>2335.12</v>
       </c>
       <c r="Q10" t="n">
-        <v>7.972</v>
+        <v>8.041</v>
       </c>
       <c r="R10" t="n">
-        <v>7.971</v>
+        <v>8.042</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1843,16 +1843,16 @@
         </is>
       </c>
       <c r="U10" t="n">
-        <v>2043.1</v>
+        <v>2132.78</v>
       </c>
       <c r="V10" t="n">
-        <v>16.36</v>
+        <v>24.47</v>
       </c>
       <c r="W10" t="n">
-        <v>1879.09</v>
+        <v>1977.32</v>
       </c>
       <c r="X10" t="n">
-        <v>147.65</v>
+        <v>130.99</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="AC10" t="n">
-        <v>411.3</v>
+        <v>419.6</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
@@ -1883,28 +1883,28 @@
         </is>
       </c>
       <c r="AE10" t="n">
-        <v>227.4</v>
+        <v>222</v>
       </c>
       <c r="AF10" t="n">
-        <v>5.89</v>
+        <v>0.8</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.641</v>
+        <v>0.248</v>
       </c>
       <c r="AH10" t="n">
-        <v>5.43</v>
+        <v>7</v>
       </c>
       <c r="AI10" t="n">
-        <v>3.22</v>
+        <v>4.79</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -1945,37 +1945,37 @@
         </is>
       </c>
       <c r="H11" s="1" t="n">
-        <v>45362</v>
+        <v>45361</v>
       </c>
       <c r="I11" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J11" t="n">
-        <v>5.600552209677709</v>
+        <v>5.60156890055749</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6018197187598008</v>
+        <v>0.6000542037503458</v>
       </c>
       <c r="L11" t="n">
-        <v>33.01</v>
+        <v>34.35</v>
       </c>
       <c r="M11" t="n">
-        <v>27.41</v>
+        <v>28.59</v>
       </c>
       <c r="N11" t="n">
-        <v>28.12</v>
+        <v>28.46</v>
       </c>
       <c r="O11" t="n">
-        <v>20.92</v>
+        <v>20.73</v>
       </c>
       <c r="P11" t="n">
-        <v>2226.06</v>
+        <v>2345.29</v>
       </c>
       <c r="Q11" t="n">
-        <v>7.954</v>
+        <v>7.978</v>
       </c>
       <c r="R11" t="n">
-        <v>7.953</v>
+        <v>7.969</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1988,16 +1988,16 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>2014.21</v>
+        <v>2081.97</v>
       </c>
       <c r="V11" t="n">
-        <v>214.12</v>
+        <v>217.25</v>
       </c>
       <c r="W11" t="n">
-        <v>1881.49</v>
+        <v>1899.33</v>
       </c>
       <c r="X11" t="n">
-        <v>118.6</v>
+        <v>165.39</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="AC11" t="n">
-        <v>406</v>
+        <v>420.6</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
@@ -2028,28 +2028,28 @@
         </is>
       </c>
       <c r="AE11" t="n">
-        <v>199.5</v>
+        <v>202.2</v>
       </c>
       <c r="AF11" t="n">
-        <v>4.08</v>
+        <v>1.24</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.12</v>
+        <v>0.99</v>
       </c>
       <c r="AH11" t="n">
-        <v>10.21</v>
+        <v>11.78</v>
       </c>
       <c r="AI11" t="n">
-        <v>4.43</v>
+        <v>0.37</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2090,37 +2090,37 @@
         </is>
       </c>
       <c r="H12" s="1" t="n">
-        <v>45406</v>
+        <v>45362</v>
       </c>
       <c r="I12" t="n">
         <v>10</v>
       </c>
       <c r="J12" t="n">
-        <v>5.646345884904603</v>
+        <v>5.653117639921701</v>
       </c>
       <c r="K12" t="n">
-        <v>0.6490489174490108</v>
+        <v>0.6491842265836193</v>
       </c>
       <c r="L12" t="n">
-        <v>33.77</v>
+        <v>34.09</v>
       </c>
       <c r="M12" t="n">
-        <v>25.62</v>
+        <v>27.03</v>
       </c>
       <c r="N12" t="n">
-        <v>25.85</v>
+        <v>27.06</v>
       </c>
       <c r="O12" t="n">
-        <v>9.59</v>
+        <v>15.35</v>
       </c>
       <c r="P12" t="n">
-        <v>2206.02</v>
+        <v>2324.59</v>
       </c>
       <c r="Q12" t="n">
-        <v>8.119</v>
+        <v>8.002000000000001</v>
       </c>
       <c r="R12" t="n">
-        <v>8.109</v>
+        <v>8.003</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -2133,16 +2133,16 @@
         </is>
       </c>
       <c r="U12" t="n">
-        <v>2014.46</v>
+        <v>2128.06</v>
       </c>
       <c r="V12" t="n">
-        <v>22.73</v>
+        <v>14.18</v>
       </c>
       <c r="W12" t="n">
-        <v>1901.03</v>
+        <v>1994.93</v>
       </c>
       <c r="X12" t="n">
-        <v>90.7</v>
+        <v>118.95</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="AC12" t="n">
-        <v>456.8</v>
+        <v>443.7</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
@@ -2173,28 +2173,28 @@
         </is>
       </c>
       <c r="AE12" t="n">
-        <v>192</v>
+        <v>235.7</v>
       </c>
       <c r="AF12" t="n">
-        <v>1.79</v>
+        <v>5.44</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.493</v>
+        <v>0.986</v>
       </c>
       <c r="AH12" t="n">
-        <v>14.42</v>
+        <v>11.24</v>
       </c>
       <c r="AI12" t="n">
-        <v>2.53</v>
+        <v>1.46</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2235,37 +2235,37 @@
         </is>
       </c>
       <c r="H13" s="1" t="n">
-        <v>45378</v>
+        <v>45363</v>
       </c>
       <c r="I13" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J13" t="n">
-        <v>5.696210316143382</v>
+        <v>5.703098212879543</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6987320948005923</v>
+        <v>0.698173305830031</v>
       </c>
       <c r="L13" t="n">
-        <v>34.69</v>
+        <v>34.33</v>
       </c>
       <c r="M13" t="n">
-        <v>24.08</v>
+        <v>27.32</v>
       </c>
       <c r="N13" t="n">
-        <v>24.65</v>
+        <v>27.18</v>
       </c>
       <c r="O13" t="n">
-        <v>9.779999999999999</v>
+        <v>18.58</v>
       </c>
       <c r="P13" t="n">
-        <v>2279.7</v>
+        <v>2229.06</v>
       </c>
       <c r="Q13" t="n">
-        <v>8.071</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="R13" t="n">
-        <v>8.074999999999999</v>
+        <v>8.073</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
         </is>
       </c>
       <c r="U13" t="n">
-        <v>2016.45</v>
+        <v>2021.2</v>
       </c>
       <c r="V13" t="n">
-        <v>12.66</v>
+        <v>18.16</v>
       </c>
       <c r="W13" t="n">
-        <v>1876.61</v>
+        <v>1919.67</v>
       </c>
       <c r="X13" t="n">
-        <v>127.18</v>
+        <v>83.37</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="AC13" t="n">
-        <v>409.3</v>
+        <v>407.2</v>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
@@ -2318,28 +2318,28 @@
         </is>
       </c>
       <c r="AE13" t="n">
-        <v>194.9</v>
+        <v>208.5</v>
       </c>
       <c r="AF13" t="n">
-        <v>6.63</v>
+        <v>1.09</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.915</v>
+        <v>0.316</v>
       </c>
       <c r="AH13" t="n">
-        <v>2.47</v>
+        <v>4.26</v>
       </c>
       <c r="AI13" t="n">
-        <v>1.54</v>
+        <v>3.57</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2380,37 +2380,37 @@
         </is>
       </c>
       <c r="H14" s="1" t="n">
-        <v>45390</v>
+        <v>45364</v>
       </c>
       <c r="I14" t="n">
         <v>2</v>
       </c>
       <c r="J14" t="n">
-        <v>5.552932349513309</v>
+        <v>5.550864371747913</v>
       </c>
       <c r="K14" t="n">
-        <v>0.5491855612291524</v>
+        <v>0.5527108357763126</v>
       </c>
       <c r="L14" t="n">
-        <v>33.25</v>
+        <v>34.11</v>
       </c>
       <c r="M14" t="n">
-        <v>25.78</v>
+        <v>27.44</v>
       </c>
       <c r="N14" t="n">
-        <v>25.41</v>
+        <v>27.19</v>
       </c>
       <c r="O14" t="n">
-        <v>14.22</v>
+        <v>22.03</v>
       </c>
       <c r="P14" t="n">
-        <v>2259.85</v>
+        <v>2211.05</v>
       </c>
       <c r="Q14" t="n">
-        <v>8.119999999999999</v>
+        <v>8.141</v>
       </c>
       <c r="R14" t="n">
-        <v>8.122999999999999</v>
+        <v>8.148999999999999</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -2423,16 +2423,16 @@
         </is>
       </c>
       <c r="U14" t="n">
-        <v>2034.53</v>
+        <v>1980.87</v>
       </c>
       <c r="V14" t="n">
-        <v>18.96</v>
+        <v>11.96</v>
       </c>
       <c r="W14" t="n">
-        <v>1929.32</v>
+        <v>1820.55</v>
       </c>
       <c r="X14" t="n">
-        <v>86.25</v>
+        <v>148.36</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="AC14" t="n">
-        <v>489.7</v>
+        <v>444.9</v>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
@@ -2463,28 +2463,28 @@
         </is>
       </c>
       <c r="AE14" t="n">
-        <v>222.9</v>
+        <v>231.8</v>
       </c>
       <c r="AF14" t="n">
-        <v>6.6</v>
+        <v>7.31</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.867</v>
+        <v>1.007</v>
       </c>
       <c r="AH14" t="n">
-        <v>5.41</v>
+        <v>4.59</v>
       </c>
       <c r="AI14" t="n">
-        <v>2.62</v>
+        <v>2.39</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2525,37 +2525,37 @@
         </is>
       </c>
       <c r="H15" s="1" t="n">
-        <v>45380</v>
+        <v>45365</v>
       </c>
       <c r="I15" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J15" t="n">
-        <v>5.599972278369346</v>
+        <v>5.599274657534936</v>
       </c>
       <c r="K15" t="n">
-        <v>0.6029629877983176</v>
+        <v>0.5999951360052959</v>
       </c>
       <c r="L15" t="n">
-        <v>35.64</v>
+        <v>35.82</v>
       </c>
       <c r="M15" t="n">
-        <v>25.48</v>
+        <v>28.26</v>
       </c>
       <c r="N15" t="n">
-        <v>25.23</v>
+        <v>28.47</v>
       </c>
       <c r="O15" t="n">
-        <v>7.2</v>
+        <v>16.2</v>
       </c>
       <c r="P15" t="n">
-        <v>2211.75</v>
+        <v>2295.45</v>
       </c>
       <c r="Q15" t="n">
-        <v>8.077999999999999</v>
+        <v>8.117000000000001</v>
       </c>
       <c r="R15" t="n">
-        <v>8.074999999999999</v>
+        <v>8.122</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -2568,16 +2568,16 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>2003.1</v>
+        <v>2109.02</v>
       </c>
       <c r="V15" t="n">
-        <v>16.87</v>
+        <v>18.65</v>
       </c>
       <c r="W15" t="n">
-        <v>1853</v>
+        <v>1977.78</v>
       </c>
       <c r="X15" t="n">
-        <v>133.23</v>
+        <v>112.59</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="AC15" t="n">
-        <v>424.3</v>
+        <v>483.5</v>
       </c>
       <c r="AD15" t="inlineStr">
         <is>
@@ -2608,28 +2608,28 @@
         </is>
       </c>
       <c r="AE15" t="n">
-        <v>194</v>
+        <v>231</v>
       </c>
       <c r="AF15" t="n">
-        <v>2.23</v>
+        <v>7.74</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.25</v>
+        <v>0.789</v>
       </c>
       <c r="AH15" t="n">
-        <v>11.12</v>
+        <v>5.06</v>
       </c>
       <c r="AI15" t="n">
-        <v>3.76</v>
+        <v>4.4</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2670,37 +2670,37 @@
         </is>
       </c>
       <c r="H16" s="1" t="n">
-        <v>45405</v>
+        <v>45366</v>
       </c>
       <c r="I16" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J16" t="n">
-        <v>5.64778586191936</v>
+        <v>5.647843494896325</v>
       </c>
       <c r="K16" t="n">
-        <v>0.6499358543408558</v>
+        <v>0.651638155136534</v>
       </c>
       <c r="L16" t="n">
-        <v>35.13</v>
+        <v>34.57</v>
       </c>
       <c r="M16" t="n">
-        <v>27.77</v>
+        <v>25.01</v>
       </c>
       <c r="N16" t="n">
-        <v>27.75</v>
+        <v>25</v>
       </c>
       <c r="O16" t="n">
-        <v>14.44</v>
+        <v>23.16</v>
       </c>
       <c r="P16" t="n">
-        <v>2326.13</v>
+        <v>2303.65</v>
       </c>
       <c r="Q16" t="n">
-        <v>8.032</v>
+        <v>8.045</v>
       </c>
       <c r="R16" t="n">
-        <v>8.032</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -2713,16 +2713,16 @@
         </is>
       </c>
       <c r="U16" t="n">
-        <v>2130.28</v>
+        <v>2111.79</v>
       </c>
       <c r="V16" t="n">
-        <v>12.6</v>
+        <v>19.7</v>
       </c>
       <c r="W16" t="n">
         <v>-50</v>
       </c>
       <c r="X16" t="n">
-        <v>136.28</v>
+        <v>148.85</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="AC16" t="n">
-        <v>480.4</v>
+        <v>397.8</v>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
@@ -2753,28 +2753,28 @@
         </is>
       </c>
       <c r="AE16" t="n">
-        <v>235.4</v>
+        <v>192.9</v>
       </c>
       <c r="AF16" t="n">
-        <v>6.74</v>
+        <v>1.5</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.279</v>
+        <v>0.695</v>
       </c>
       <c r="AH16" t="n">
-        <v>7.92</v>
+        <v>10.82</v>
       </c>
       <c r="AI16" t="n">
-        <v>4.07</v>
+        <v>0.43</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2815,37 +2815,37 @@
         </is>
       </c>
       <c r="H17" s="1" t="n">
-        <v>45401</v>
+        <v>45367</v>
       </c>
       <c r="I17" t="n">
         <v>20</v>
       </c>
       <c r="J17" t="n">
-        <v>5.69746481053699</v>
+        <v>5.699689096762078</v>
       </c>
       <c r="K17" t="n">
-        <v>0.7007394496986431</v>
+        <v>0.701576438730213</v>
       </c>
       <c r="L17" t="n">
-        <v>33.99</v>
+        <v>34.16</v>
       </c>
       <c r="M17" t="n">
-        <v>27.54</v>
+        <v>28.68</v>
       </c>
       <c r="N17" t="n">
-        <v>27.43</v>
+        <v>28.87</v>
       </c>
       <c r="O17" t="n">
-        <v>21.85</v>
+        <v>22.34</v>
       </c>
       <c r="P17" t="n">
-        <v>2331.94</v>
+        <v>2277.49</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.054</v>
+        <v>8.003</v>
       </c>
       <c r="R17" t="n">
-        <v>8.058</v>
+        <v>8.01</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2858,16 +2858,16 @@
         </is>
       </c>
       <c r="U17" t="n">
-        <v>2099.73</v>
+        <v>2090.22</v>
       </c>
       <c r="V17" t="n">
-        <v>15.09</v>
+        <v>20.94</v>
       </c>
       <c r="W17" t="n">
-        <v>1992.07</v>
+        <v>1973.22</v>
       </c>
       <c r="X17" t="n">
-        <v>92.56999999999999</v>
+        <v>96.06</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="AC17" t="n">
-        <v>478.3</v>
+        <v>385.3</v>
       </c>
       <c r="AD17" t="inlineStr">
         <is>
@@ -2898,28 +2898,28 @@
         </is>
       </c>
       <c r="AE17" t="n">
-        <v>238.3</v>
+        <v>200</v>
       </c>
       <c r="AF17" t="n">
-        <v>5.32</v>
+        <v>3.09</v>
       </c>
       <c r="AG17" t="n">
-        <v>0.321</v>
+        <v>0.948</v>
       </c>
       <c r="AH17" t="n">
-        <v>13.39</v>
+        <v>14.74</v>
       </c>
       <c r="AI17" t="n">
-        <v>3.09</v>
+        <v>1.22</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -2960,37 +2960,37 @@
         </is>
       </c>
       <c r="H18" s="1" t="n">
-        <v>45374</v>
+        <v>45368</v>
       </c>
       <c r="I18" t="n">
         <v>2</v>
       </c>
       <c r="J18" t="n">
-        <v>5.551110715903227</v>
+        <v>5.548638105903003</v>
       </c>
       <c r="K18" t="n">
-        <v>0.5519965120783518</v>
+        <v>0.5501601379967801</v>
       </c>
       <c r="L18" t="n">
-        <v>33.08</v>
+        <v>35.96</v>
       </c>
       <c r="M18" t="n">
-        <v>27.16</v>
+        <v>26.85</v>
       </c>
       <c r="N18" t="n">
-        <v>27.47</v>
+        <v>26.81</v>
       </c>
       <c r="O18" t="n">
-        <v>5.42</v>
+        <v>21.36</v>
       </c>
       <c r="P18" t="n">
-        <v>2259.84</v>
+        <v>2261.61</v>
       </c>
       <c r="Q18" t="n">
-        <v>8.099</v>
+        <v>7.972</v>
       </c>
       <c r="R18" t="n">
-        <v>8.101000000000001</v>
+        <v>7.971</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
         </is>
       </c>
       <c r="U18" t="n">
-        <v>1991.87</v>
+        <v>2043.1</v>
       </c>
       <c r="V18" t="n">
-        <v>10.46</v>
+        <v>16.36</v>
       </c>
       <c r="W18" t="n">
-        <v>1886.56</v>
+        <v>1879.09</v>
       </c>
       <c r="X18" t="n">
-        <v>94.84999999999999</v>
+        <v>147.65</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="AC18" t="n">
-        <v>387</v>
+        <v>485.2</v>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
@@ -3043,28 +3043,28 @@
         </is>
       </c>
       <c r="AE18" t="n">
-        <v>196.7</v>
+        <v>218.3</v>
       </c>
       <c r="AF18" t="n">
-        <v>4.71</v>
+        <v>4.51</v>
       </c>
       <c r="AG18" t="n">
-        <v>0.83</v>
+        <v>0.163</v>
       </c>
       <c r="AH18" t="n">
-        <v>2.63</v>
+        <v>11.88</v>
       </c>
       <c r="AI18" t="n">
-        <v>4.48</v>
+        <v>1.02</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -3105,37 +3105,37 @@
         </is>
       </c>
       <c r="H19" s="1" t="n">
-        <v>45397</v>
+        <v>45369</v>
       </c>
       <c r="I19" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J19" t="n">
-        <v>5.602360228580113</v>
+        <v>5.600552209677709</v>
       </c>
       <c r="K19" t="n">
-        <v>0.6039880178887252</v>
+        <v>0.6018197187598008</v>
       </c>
       <c r="L19" t="n">
-        <v>33.13</v>
+        <v>33.01</v>
       </c>
       <c r="M19" t="n">
-        <v>25.74</v>
+        <v>27.41</v>
       </c>
       <c r="N19" t="n">
-        <v>26.24</v>
+        <v>28.12</v>
       </c>
       <c r="O19" t="n">
-        <v>3.01</v>
+        <v>13.09</v>
       </c>
       <c r="P19" t="n">
-        <v>2248.98</v>
+        <v>2226.06</v>
       </c>
       <c r="Q19" t="n">
-        <v>8.013999999999999</v>
+        <v>7.954</v>
       </c>
       <c r="R19" t="n">
-        <v>8.023</v>
+        <v>7.953</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -3148,16 +3148,16 @@
         </is>
       </c>
       <c r="U19" t="n">
-        <v>1990.06</v>
+        <v>2014.21</v>
       </c>
       <c r="V19" t="n">
-        <v>13.84</v>
+        <v>14.12</v>
       </c>
       <c r="W19" t="n">
-        <v>1841.28</v>
+        <v>1881.49</v>
       </c>
       <c r="X19" t="n">
-        <v>134.94</v>
+        <v>118.6</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -3180,7 +3180,7 @@
         </is>
       </c>
       <c r="AC19" t="n">
-        <v>404</v>
+        <v>417</v>
       </c>
       <c r="AD19" t="inlineStr">
         <is>
@@ -3188,28 +3188,28 @@
         </is>
       </c>
       <c r="AE19" t="n">
-        <v>207.3</v>
+        <v>220.4</v>
       </c>
       <c r="AF19" t="n">
-        <v>6.36</v>
+        <v>5.81</v>
       </c>
       <c r="AG19" t="n">
-        <v>1.177</v>
+        <v>0.948</v>
       </c>
       <c r="AH19" t="n">
-        <v>4.75</v>
+        <v>14.19</v>
       </c>
       <c r="AI19" t="n">
-        <v>4.6</v>
+        <v>2.92</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -3250,37 +3250,37 @@
         </is>
       </c>
       <c r="H20" s="1" t="n">
-        <v>45407</v>
+        <v>45370</v>
       </c>
       <c r="I20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J20" t="n">
-        <v>5.651013815401549</v>
+        <v>5.646345884904603</v>
       </c>
       <c r="K20" t="n">
-        <v>0.6480005040258755</v>
+        <v>0.6490489174490108</v>
       </c>
       <c r="L20" t="n">
-        <v>34.76</v>
+        <v>33.77</v>
       </c>
       <c r="M20" t="n">
-        <v>28.6</v>
+        <v>25.62</v>
       </c>
       <c r="N20" t="n">
-        <v>28.8</v>
+        <v>25.85</v>
       </c>
       <c r="O20" t="n">
-        <v>22.16</v>
+        <v>17.19</v>
       </c>
       <c r="P20" t="n">
-        <v>2207.42</v>
+        <v>2206.02</v>
       </c>
       <c r="Q20" t="n">
-        <v>8.057</v>
+        <v>8.119</v>
       </c>
       <c r="R20" t="n">
-        <v>8.050000000000001</v>
+        <v>8.109</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -3293,16 +3293,16 @@
         </is>
       </c>
       <c r="U20" t="n">
-        <v>2014.89</v>
+        <v>2014.46</v>
       </c>
       <c r="V20" t="n">
-        <v>12.3</v>
+        <v>22.73</v>
       </c>
       <c r="W20" t="n">
-        <v>1900.18</v>
+        <v>1901.03</v>
       </c>
       <c r="X20" t="n">
-        <v>102.41</v>
+        <v>90.7</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="AC20" t="n">
-        <v>447.9</v>
+        <v>442.8</v>
       </c>
       <c r="AD20" t="inlineStr">
         <is>
@@ -3333,28 +3333,28 @@
         </is>
       </c>
       <c r="AE20" t="n">
-        <v>216.7</v>
+        <v>194.6</v>
       </c>
       <c r="AF20" t="n">
-        <v>1.24</v>
+        <v>5.41</v>
       </c>
       <c r="AG20" t="n">
-        <v>0.924</v>
+        <v>0.982</v>
       </c>
       <c r="AH20" t="n">
-        <v>4.23</v>
+        <v>10.6</v>
       </c>
       <c r="AI20" t="n">
-        <v>3.06</v>
+        <v>2.95</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -3395,37 +3395,37 @@
         </is>
       </c>
       <c r="H21" s="1" t="n">
-        <v>45364</v>
+        <v>45371</v>
       </c>
       <c r="I21" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J21" t="n">
-        <v>5.700914930522096</v>
+        <v>5.696210316143382</v>
       </c>
       <c r="K21" t="n">
-        <v>0.7014779742688503</v>
+        <v>0.6987320948005923</v>
       </c>
       <c r="L21" t="n">
-        <v>34.23</v>
+        <v>34.69</v>
       </c>
       <c r="M21" t="n">
-        <v>25.05</v>
+        <v>24.08</v>
       </c>
       <c r="N21" t="n">
-        <v>24.98</v>
+        <v>24.65</v>
       </c>
       <c r="O21" t="n">
-        <v>9.09</v>
+        <v>23.11</v>
       </c>
       <c r="P21" t="n">
-        <v>2264.43</v>
+        <v>2279.7</v>
       </c>
       <c r="Q21" t="n">
-        <v>8.085000000000001</v>
+        <v>8.071</v>
       </c>
       <c r="R21" t="n">
-        <v>8.082000000000001</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -3438,16 +3438,16 @@
         </is>
       </c>
       <c r="U21" t="n">
-        <v>2041.37</v>
+        <v>2016.45</v>
       </c>
       <c r="V21" t="n">
-        <v>23.41</v>
+        <v>12.66</v>
       </c>
       <c r="W21" t="n">
-        <v>1896.91</v>
+        <v>1876.61</v>
       </c>
       <c r="X21" t="n">
-        <v>121.05</v>
+        <v>127.18</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="AC21" t="n">
-        <v>453</v>
+        <v>470.9</v>
       </c>
       <c r="AD21" t="inlineStr">
         <is>
@@ -3478,28 +3478,28 @@
         </is>
       </c>
       <c r="AE21" t="n">
-        <v>225.4</v>
+        <v>206.1</v>
       </c>
       <c r="AF21" t="n">
-        <v>6.36</v>
+        <v>6.97</v>
       </c>
       <c r="AG21" t="n">
-        <v>1.129</v>
+        <v>1.14</v>
       </c>
       <c r="AH21" t="n">
-        <v>9.369999999999999</v>
+        <v>13.95</v>
       </c>
       <c r="AI21" t="n">
-        <v>1.52</v>
+        <v>0.67</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>PyCO2SYS</t>
+          <t>synthetic_example_generator</t>
         </is>
       </c>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>TA + pH_observed</t>
+          <t>synthetic TA + pH_observed</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
         <v>35</v>
       </c>
       <c r="M22" t="n">
-        <v>25.2</v>
+        <v>25.41</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
@@ -3545,7 +3545,7 @@
         <v>2204.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>8.050000000000001</v>
+        <v>8.061999999999999</v>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
@@ -3610,7 +3610,7 @@
         <v>35</v>
       </c>
       <c r="M23" t="n">
-        <v>25.25</v>
+        <v>25.31</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
@@ -3618,7 +3618,7 @@
         <v>2202.8</v>
       </c>
       <c r="Q23" t="n">
-        <v>8.085000000000001</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr">
@@ -3683,7 +3683,7 @@
         <v>35</v>
       </c>
       <c r="M24" t="n">
-        <v>25.03</v>
+        <v>25.48</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
         <v>2208.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>8.068</v>
+        <v>8.081</v>
       </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
@@ -3756,7 +3756,7 @@
         <v>35</v>
       </c>
       <c r="M25" t="n">
-        <v>25.2</v>
+        <v>25.29</v>
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
@@ -3764,7 +3764,7 @@
         <v>2203.6</v>
       </c>
       <c r="Q25" t="n">
-        <v>8.096</v>
+        <v>8.093999999999999</v>
       </c>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">

</xml_diff>

<commit_message>
Initial commit: oa_pipeline v0.2.0
</commit_message>
<xml_diff>
--- a/examples/example_data.xlsx
+++ b/examples/example_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="oa_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="oa_data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,187 +433,187 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>sample_tag</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>crm_or_sample</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sample_id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>cruise_id</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>transect_id</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>station_id</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>replicate_id</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>sample_date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>depth_m</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>latitude_deg</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>longitude_deg</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>salinity</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>temp_lab</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>temperature_insitu_c</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>pressure_output_dbar</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>pH_lab</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ph_calculated</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>ph_scale_observed</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>ph_scale_calculated</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>dic_calculated_umol_kg</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>co2aq_calc_umol_kg</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>hco3_calc_umol_kg</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>co3_calc_umol_kg</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>dic_unit</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>co2aq_unit</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>hco3_unit</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>co3_unit</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>pco2_calc_uatm</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>ta_units</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>oxygen_umol_l</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>nitrate_nitrite_umol_l</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>phosphate_umol_l</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>silicate_umol_l</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>chlorophyll</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>carbonate_solver</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>carbon_input_pair_used</t>
         </is>
@@ -643,7 +655,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="I2" t="n">
@@ -788,7 +800,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>45353</v>
       </c>
       <c r="I3" t="n">
@@ -933,7 +945,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>45354</v>
       </c>
       <c r="I4" t="n">
@@ -1078,7 +1090,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>45355</v>
       </c>
       <c r="I5" t="n">
@@ -1223,7 +1235,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>45356</v>
       </c>
       <c r="I6" t="n">
@@ -1368,7 +1380,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>45357</v>
       </c>
       <c r="I7" t="n">
@@ -1509,7 +1521,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>45358</v>
       </c>
       <c r="I8" t="n">
@@ -1654,7 +1666,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>45359</v>
       </c>
       <c r="I9" t="n">
@@ -1799,7 +1811,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>45360</v>
       </c>
       <c r="I10" t="n">
@@ -1944,7 +1956,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>45361</v>
       </c>
       <c r="I11" t="n">
@@ -2089,7 +2101,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>45362</v>
       </c>
       <c r="I12" t="n">
@@ -2234,7 +2246,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>45363</v>
       </c>
       <c r="I13" t="n">
@@ -2379,7 +2391,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>45364</v>
       </c>
       <c r="I14" t="n">
@@ -2524,7 +2536,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>45365</v>
       </c>
       <c r="I15" t="n">
@@ -2669,7 +2681,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I16" t="n">
@@ -2814,7 +2826,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>45367</v>
       </c>
       <c r="I17" t="n">
@@ -2959,7 +2971,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>45368</v>
       </c>
       <c r="I18" t="n">
@@ -3104,7 +3116,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>45369</v>
       </c>
       <c r="I19" t="n">
@@ -3249,7 +3261,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>45370</v>
       </c>
       <c r="I20" t="n">
@@ -3394,7 +3406,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>45371</v>
       </c>
       <c r="I21" t="n">
@@ -3527,7 +3539,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -3600,7 +3612,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -3673,7 +3685,7 @@
           <t>r3</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -3746,7 +3758,7 @@
           <t>r4</t>
         </is>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -3819,7 +3831,7 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -3886,7 +3898,7 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -3953,7 +3965,7 @@
           <t>r3</t>
         </is>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="I28" t="inlineStr"/>

</xml_diff>